<commit_message>
Se agregan requirements.txt y dotenv
</commit_message>
<xml_diff>
--- a/Planilla_Oficial_Rodeo.xlsx
+++ b/Planilla_Oficial_Rodeo.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,37 +433,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>club_organizador</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>contacto</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>criadero</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>serie</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>binomios</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>fecha_registro</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>estado</t>
         </is>
@@ -483,7 +495,7 @@
           <t>[{'jinete': 'Alejandro Varela', 'rut': '6.448.321-8', 'club_origen': 'Club Cordillera', 'caballo': 'Huacha soy', 'cod_caballo': 238972}, {'jinete': 'Pablo Barra', 'rut': '12.369.452-k', 'club_origen': 'Club Cordillera', 'caballo': 'Esperada', 'cod_caballo': 230210}]</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>46142.41666666666</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,7 +530,7 @@
           <t>[{'jinete': 'Rodrigo Fontecilla', 'rut': '15.314.315-3', 'club_origen': 'Invitado', 'caballo': 'Gallo Pulento', 'cod_caballo': 271652}, {'jinete': 'Julián Calderón', 'rut': '17.811.134-5', 'club_origen': 'Invitado', 'caballo': 'Galla Encantada', 'cod_caballo': 271654}]</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>46143.47916666666</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -553,7 +565,7 @@
           <t>[{'jinete': 'Sebastian Varela', 'rut': '16.662.180-1', 'club_origen': 'las vizcachas de puente alto', 'caballo': 'Princesa', 'cod_caballo': 235703}, {'jinete': 'Leonardo Espinoza', 'rut': '10.752.940-3', 'club_origen': 'Club Pirque', 'caballo': 'Chunteria', 'cod_caballo': 255488}]</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>46143.58333333334</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -588,7 +600,7 @@
           <t>[{'jinete': 'Max Bravo', 'rut': '10.253.941-9', 'club_origen': 'Club Rio Maipo', 'caballo': 'Ilusion', 'cod_caballo': 283897}, {'jinete': 'José Flores', 'rut': '17.544.248-0', 'club_origen': 'Club Rio Maipo', 'caballo': 'Empeñosa', 'cod_caballo': 283896}]</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>46144.375</v>
       </c>
       <c r="G5" t="inlineStr">
@@ -623,7 +635,7 @@
           <t>[{'jinete': 'Francisco Moraga', 'rut': '10.518.993-1', 'club_origen': 'Invitado', 'caballo': 'Ladino', 'cod_caballo': 255339}, {'jinete': 'Diego Moraga', 'rut': '13.068.291-0', 'club_origen': 'Invitado', 'caballo': 'Escogida', 'cod_caballo': 259848}]</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>46144.42708333334</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -658,7 +670,7 @@
           <t>[{'jinete': 'Emiliano Ruiz', 'rut': '23.431.238-3', 'club_origen': 'Invitado', 'caballo': 'Orgullo', 'cod_caballo': 245756}, {'jinete': 'Emiliano Ruiz (h)', 'rut': '13.252.337-1', 'club_origen': 'Invitado', 'caballo': 'Candidato', 'cod_caballo': 234632}]</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>46145.35416666666</v>
       </c>
       <c r="G7" t="inlineStr">
@@ -693,7 +705,7 @@
           <t>[{'jinete': 'Juan Perez', 'rut': '14.123.456-7', 'club_origen': 'Club San José', 'caballo': 'Relámpago', 'cod_caballo': 290123}, {'jinete': 'Luis Soto', 'rut': '15.987.654-3', 'club_origen': 'Club San José', 'caballo': 'Tormenta', 'cod_caballo': 290124}]</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>46145.5</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -728,7 +740,7 @@
           <t>[{'jinete': 'Carlos Rivas', 'rut': '11.222.333-4', 'club_origen': 'Club Pirque', 'caballo': 'Estruendo', 'cod_caballo': 299444}, {'jinete': 'Miguel Rivas', 'rut': '18.333.444-5', 'club_origen': 'Club Pirque', 'caballo': 'Chispa', 'cod_caballo': 299445}]</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>46146.40625</v>
       </c>
       <c r="G9" t="inlineStr">
@@ -763,7 +775,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>46155.92457594907</v>
       </c>
       <c r="G10" t="inlineStr">

</xml_diff>

<commit_message>
Modificaciones a menus, exportacion ahora es opcional, readme pendiente de actualizacion
</commit_message>
<xml_diff>
--- a/Planilla_Oficial_Rodeo.xlsx
+++ b/Planilla_Oficial_Rodeo.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -784,6 +784,41 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Club El Rodeo</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>{'nombre': 'Juan Perez', 'fono': '56912345678', 'email': 's/i'}</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Los Aromos</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[{'jinete': 'Pedro Gonzalez', 'rut': '12345678-9', 'caballo': 'Relampago', 'club_origen': 'Club El Rodeo'}, {'jinete': 'Maria Silva', 'rut': '98765432-1', 'caballo': 'Centella', 'club_origen': 'Club El Rodeo'}]</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>46156.98593836805</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>